<commit_message>
use one led that blinks on alarm since we only have a green one
</commit_message>
<xml_diff>
--- a/BOM_pico_serverrum.xlsx
+++ b/BOM_pico_serverrum.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -640,21 +640,21 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Visar direkt på enheten att klimatet är OK, så personal ser status utan att öppna Grafana.</t>
+          <t>Statuslampa direkt på enheten. Lyser fast när klimatet är OK och blinkar vid larm, så personal ser läget utan att öppna Grafana.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Lysdiod 5mm röd</t>
+          <t>Motstånd 330 ohm</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D8" s="6">
         <f>B8*$B$2</f>
@@ -666,26 +666,26 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/led-5mm-rod-diffus</t>
+          <t>https://www.electrokit.com/motstand-kolfilm-0.25w-330ohm-330r</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Larmindikator som tänds lokalt när temperatur eller fuktighet går över gränsvärdet.</t>
+          <t>Strömbegränsar lysdioden så att varken dioden eller GPIO-pinnen blir förstörd.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Motstånd 330 ohm</t>
+          <t>Kopplingsdäck 830 hål</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="D9" s="6">
         <f>B9*$B$2</f>
@@ -697,26 +697,26 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/motstand-kolfilm-0.25w-330ohm-330r</t>
+          <t>https://www.electrokit.com/kopplingsdack-830-anslutningar</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Strömbegränsar lysdioderna så att varken dioderna eller GPIO-pinnarna blir förstörda.</t>
+          <t>Gör att vi kan koppla prototypen utan att löda och snabbt kan ändra kopplingen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Kopplingsdäck 830 hål</t>
+          <t>Kopplingskablar hane-hane 40-pack</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="D10" s="6">
         <f>B10*$B$2</f>
@@ -728,26 +728,26 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/kopplingsdack-830-anslutningar</t>
+          <t>https://www.electrokit.com/labbsladd-40-pin-hane-hane-150mm</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>Gör att vi kan koppla prototypen utan att löda och snabbt kan ändra kopplingen.</t>
+          <t>Behövs för att koppla ihop sensor och lysdioder med Pico:ns GPIO-pinnar.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Kopplingskablar hane-hane 40-pack</t>
+          <t>USB-kabel A - micro B</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D11" s="6">
         <f>B11*$B$2</f>
@@ -759,80 +759,49 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/labbsladd-40-pin-hane-hane-150mm</t>
+          <t>https://www.electrokit.com/usb-kabel-a-hane-micro-b-hane-1.8m</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Behövs för att koppla ihop sensor och lysdioder med Pico:ns GPIO-pinnar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>USB-kabel A - micro B</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="D12" s="6">
-        <f>B12*$B$2</f>
-        <v/>
-      </c>
-      <c r="E12" s="7">
-        <f>D12*C12</f>
-        <v/>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/usb-kabel-a-hane-micro-b-hane-1.8m</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
           <t>Ger ström till Pico:n och används för att ladda upp koden från VS Code.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>TOTALT</t>
         </is>
       </c>
-      <c r="B13" s="10">
-        <f>SUM(B5:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="10">
-        <f>SUM(D5:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="12">
-        <f>SUM(E5:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="B12" s="10">
+        <f>SUM(B5:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="10">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>SUM(E5:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Totalt antal komponenter och total kostnad för alla prototyper</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Kostnad per prototyp</t>
         </is>
       </c>
-      <c r="E15" s="13">
-        <f>E13/B2</f>
+      <c r="E14" s="13">
+        <f>E12/B2</f>
         <v/>
       </c>
     </row>
@@ -845,7 +814,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
bom with what we actually bought and paid
</commit_message>
<xml_diff>
--- a/BOM_pico_serverrum.xlsx
+++ b/BOM_pico_serverrum.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ur kitet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0 kr"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +46,10 @@
     <font>
       <color rgb="000563C1"/>
       <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +120,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,16 +486,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="68" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +512,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -551,17 +557,17 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="46" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Pi Pico 2 W</t>
+          <t>Freenove Basic Starter Kit for Raspberry Pi Pico 2 W</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>89</v>
+        <v>390</v>
       </c>
       <c r="D5" s="6">
         <f>B5*$B$2</f>
@@ -573,26 +579,26 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/raspberry-pi-pico-2-w</t>
+          <t>https://www.amazon.se/dp/B0DRJV9JJW</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Mikrokontrollern som kör MicroPython. Har inbyggt WiFi så den kan skicka mätvärden över MQTT utan extra hårdvara.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
+          <t>Kitet innehåller Pico 2 W, kopplingsdäck, kopplingskablar, lysdioder, motstånd och USB-kabel. Billigare än att köpa delarna var för sig, och vi får med reservdelar om något går sönder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>DHT11 temp- och fuktsensor (KY-015)</t>
+          <t>AZDelivery KY-015 DHT11 temperatursensormodul</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>49</v>
+        <v>129</v>
       </c>
       <c r="D6" s="6">
         <f>B6*$B$2</f>
@@ -604,204 +610,87 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://www.electrokit.com/temperatur-och-fuktsensor-dht11</t>
+          <t>https://www.amazon.se/dp/B089W8DB5P</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Mäter både temperatur och luftfuktighet, vilket är precis de två värden vi övervakar i serverrummet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Lysdiod 5mm grön</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" s="6">
-        <f>B7*$B$2</f>
-        <v/>
-      </c>
-      <c r="E7" s="7">
-        <f>D7*C7</f>
-        <v/>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/led-5mm-gron-diffus</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Statuslampa direkt på enheten. Lyser fast när klimatet är OK och blinkar vid larm, så personal ser läget utan att öppna Grafana.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>Mäter både temperatur och luftfuktighet, vilket är precis de två värden vi övervakar. Ingår inte i kitet. Modulen har motståndet inbyggt så den kan kopplas direkt till en GPIO-pinne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Summa komponenter</t>
+        </is>
+      </c>
+      <c r="B7" s="10">
+        <f>SUM(B5:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="10">
+        <f>SUM(D5:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="12">
+        <f>SUM(E5:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Totalt antal komponenter och kostnad för alla prototyper</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Motstånd 330 ohm</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>1</v>
-      </c>
+          <t>Frakt</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="6">
-        <f>B8*$B$2</f>
-        <v/>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="7">
-        <f>D8*C8</f>
-        <v/>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/motstand-kolfilm-0.25w-330ohm-330r</t>
-        </is>
-      </c>
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Strömbegränsar lysdioden så att varken dioden eller GPIO-pinnen blir förstörd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Kopplingsdäck 830 hål</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>69</v>
-      </c>
-      <c r="D9" s="6">
-        <f>B9*$B$2</f>
-        <v/>
-      </c>
-      <c r="E9" s="7">
-        <f>D9*C9</f>
-        <v/>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/kopplingsdack-830-anslutningar</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Gör att vi kan koppla prototypen utan att löda och snabbt kan ändra kopplingen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Kopplingskablar hane-hane 40-pack</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>39</v>
-      </c>
-      <c r="D10" s="6">
-        <f>B10*$B$2</f>
-        <v/>
-      </c>
-      <c r="E10" s="7">
-        <f>D10*C10</f>
-        <v/>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/labbsladd-40-pin-hane-hane-150mm</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Behövs för att koppla ihop sensor och lysdioder med Pico:ns GPIO-pinnar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>USB-kabel A - micro B</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="D11" s="6">
-        <f>B11*$B$2</f>
-        <v/>
-      </c>
-      <c r="E11" s="7">
-        <f>D11*C11</f>
-        <v/>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.electrokit.com/usb-kabel-a-hane-micro-b-hane-1.8m</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Ger ström till Pico:n och används för att ladda upp koden från VS Code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>TOTALT</t>
-        </is>
-      </c>
-      <c r="B12" s="10">
-        <f>SUM(B5:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="10">
-        <f>SUM(D5:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="12">
-        <f>SUM(E5:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>Totalt antal komponenter och total kostnad för alla prototyper</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+          <t>Engångskostnad per beställning. Växer inte med antalet prototyper eftersom allt kan beställas i samma order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TOTALT INKLUSIVE FRAKT</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="12">
+        <f>E7+E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Kostnad per prototyp</t>
         </is>
       </c>
-      <c r="E14" s="13">
-        <f>E12/B2</f>
+      <c r="E11" s="13">
+        <f>E9/B2</f>
         <v/>
       </c>
     </row>
@@ -809,12 +698,183 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Delar ur Freenove-kitet som vi använder i prototypen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Resten av kitets 142 komponenter används inte i den här produkten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Del</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Antal</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Ansluten till</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Motivering</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi Pico 2 W</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Mikrokontrollern som kör MicroPython. Har inbyggt wifi så den kan skicka mätvärden över MQTT utan extra hårdvara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Kopplingsdäck</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Gör att vi kan koppla prototypen utan att löda och snabbt ändra kopplingen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Kopplingskablar hane-hane</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Kopplar sensorn och lysdioden till Pico:ns pinnar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Lysdiod, grön</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>GP15 via motstånd</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Statuslampa direkt på enheten. Lyser fast när klimatet är OK och blinkar vid larm, så personal ser läget utan att öppna Grafana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Motstånd 330 ohm</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Mellan GP15 och lysdioden</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Strömbegränsar lysdioden så att varken dioden eller GPIO-pinnen blir förstörd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>USB-kabel</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Ger ström till Pico:n och används för att ladda upp koden från VS Code.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>